<commit_message>
deleted and modified files as a consequence of updates to fit LUCAS 2009 data import
</commit_message>
<xml_diff>
--- a/lucas/import_data/utility/observation/excel/provision_indicator.xlsx
+++ b/lucas/import_data/utility/observation/excel/provision_indicator.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="178">
   <si>
     <t xml:space="preserve">provision_id__provision_name</t>
   </si>
@@ -125,6 +125,9 @@
   </si>
   <si>
     <t xml:space="preserve">c-org iso 10694:1995</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g*kg^-1</t>
   </si>
   <si>
     <t xml:space="preserve">p-ext</t>
@@ -766,37 +769,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -870,7 +873,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1048576"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="32.65"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="31.23"/>
@@ -1113,7 +1116,7 @@
         <v>34</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1121,13 +1124,13 @@
         <v>15</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1135,13 +1138,13 @@
         <v>15</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1149,13 +1152,13 @@
         <v>15</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1163,10 +1166,10 @@
         <v>15</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>18</v>
@@ -1177,10 +1180,10 @@
         <v>15</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>18</v>
@@ -1191,18 +1194,18 @@
         <v>15</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>16</v>
@@ -1216,7 +1219,7 @@
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>19</v>
@@ -1230,7 +1233,7 @@
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>22</v>
@@ -1244,13 +1247,13 @@
     </row>
     <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>18</v>
@@ -1258,7 +1261,7 @@
     </row>
     <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>26</v>
@@ -1272,7 +1275,7 @@
     </row>
     <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>29</v>
@@ -1286,7 +1289,7 @@
     </row>
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>31</v>
@@ -1300,7 +1303,7 @@
     </row>
     <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>33</v>
@@ -1314,55 +1317,55 @@
     </row>
     <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B34" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>18</v>
@@ -1370,13 +1373,13 @@
     </row>
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>18</v>
@@ -1384,377 +1387,377 @@
     </row>
     <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B42" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D42" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>26</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D47" s="1" t="s">
         <v>67</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B49" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C49" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C49" s="1" t="s">
-        <v>71</v>
-      </c>
       <c r="D49" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D53" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C53" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D53" s="1" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D54" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="B54" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D54" s="1" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D55" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="B55" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B57" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D57" s="1" t="s">
         <v>83</v>
-      </c>
-      <c r="C57" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="D57" s="1" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D63" s="1" t="s">
         <v>7</v>
@@ -1762,13 +1765,13 @@
     </row>
     <row r="64" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B64" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C64" s="1" t="s">
         <v>97</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>96</v>
       </c>
       <c r="D64" s="1" t="s">
         <v>7</v>
@@ -1776,13 +1779,13 @@
     </row>
     <row r="65" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D65" s="1" t="s">
         <v>7</v>
@@ -1790,13 +1793,13 @@
     </row>
     <row r="66" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D66" s="1" t="s">
         <v>7</v>
@@ -1804,13 +1807,13 @@
     </row>
     <row r="67" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D67" s="1" t="s">
         <v>7</v>
@@ -1818,13 +1821,13 @@
     </row>
     <row r="68" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D68" s="1" t="s">
         <v>7</v>
@@ -1832,13 +1835,13 @@
     </row>
     <row r="69" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D69" s="1" t="s">
         <v>7</v>
@@ -1846,13 +1849,13 @@
     </row>
     <row r="70" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B70" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C70" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="C70" s="1" t="s">
-        <v>103</v>
       </c>
       <c r="D70" s="1" t="s">
         <v>7</v>
@@ -1860,13 +1863,13 @@
     </row>
     <row r="71" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D71" s="1" t="s">
         <v>7</v>
@@ -1874,13 +1877,13 @@
     </row>
     <row r="72" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D72" s="1" t="s">
         <v>7</v>
@@ -1888,13 +1891,13 @@
     </row>
     <row r="73" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B73" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C73" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="C73" s="1" t="s">
-        <v>107</v>
       </c>
       <c r="D73" s="1" t="s">
         <v>7</v>
@@ -1902,13 +1905,13 @@
     </row>
     <row r="74" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D74" s="1" t="s">
         <v>7</v>
@@ -1916,13 +1919,13 @@
     </row>
     <row r="75" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D75" s="1" t="s">
         <v>7</v>
@@ -1930,13 +1933,13 @@
     </row>
     <row r="76" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D76" s="1" t="s">
         <v>7</v>
@@ -1944,13 +1947,13 @@
     </row>
     <row r="77" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D77" s="1" t="s">
         <v>7</v>
@@ -1958,13 +1961,13 @@
     </row>
     <row r="78" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D78" s="1" t="s">
         <v>7</v>
@@ -1972,13 +1975,13 @@
     </row>
     <row r="79" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B79" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C79" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="C79" s="1" t="s">
-        <v>114</v>
       </c>
       <c r="D79" s="1" t="s">
         <v>7</v>
@@ -1986,13 +1989,13 @@
     </row>
     <row r="80" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D80" s="1" t="s">
         <v>7</v>
@@ -2000,13 +2003,13 @@
     </row>
     <row r="81" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D81" s="1" t="s">
         <v>7</v>
@@ -2014,125 +2017,125 @@
     </row>
     <row r="82" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D90" s="1" t="s">
         <v>7</v>
@@ -2140,13 +2143,13 @@
     </row>
     <row r="91" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D91" s="1" t="s">
         <v>7</v>
@@ -2154,7 +2157,7 @@
     </row>
     <row r="92" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B92" s="1" t="s">
         <v>8</v>
@@ -2168,7 +2171,7 @@
     </row>
     <row r="93" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B93" s="1" t="s">
         <v>5</v>
@@ -2182,7 +2185,7 @@
     </row>
     <row r="94" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B94" s="1" t="s">
         <v>10</v>
@@ -2196,7 +2199,7 @@
     </row>
     <row r="95" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B95" s="1" t="s">
         <v>12</v>
@@ -2210,7 +2213,7 @@
     </row>
     <row r="96" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B96" s="1" t="s">
         <v>8</v>
@@ -2224,7 +2227,7 @@
     </row>
     <row r="97" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B97" s="1" t="s">
         <v>5</v>
@@ -2238,7 +2241,7 @@
     </row>
     <row r="98" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B98" s="1" t="s">
         <v>10</v>
@@ -2252,7 +2255,7 @@
     </row>
     <row r="99" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B99" s="1" t="s">
         <v>12</v>
@@ -2266,21 +2269,21 @@
     </row>
     <row r="100" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B100" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D100" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="C100" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D100" s="1" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B101" s="1" t="s">
         <v>26</v>
@@ -2289,12 +2292,12 @@
         <v>27</v>
       </c>
       <c r="D101" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B102" s="1" t="s">
         <v>33</v>
@@ -2308,7 +2311,7 @@
     </row>
     <row r="103" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B103" s="1" t="s">
         <v>31</v>
@@ -2322,63 +2325,63 @@
     </row>
     <row r="104" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C104" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D104" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B105" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C105" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="D105" s="1" t="s">
         <v>141</v>
-      </c>
-      <c r="C105" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D105" s="1" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C106" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D106" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C107" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D107" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B108" s="1" t="s">
         <v>19</v>
@@ -2387,32 +2390,32 @@
         <v>20</v>
       </c>
       <c r="D108" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D109" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B110" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D110" s="1" t="s">
         <v>18</v>
@@ -2420,13 +2423,13 @@
     </row>
     <row r="111" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D111" s="1" t="s">
         <v>18</v>
@@ -2434,13 +2437,13 @@
     </row>
     <row r="112" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D112" s="1" t="s">
         <v>18</v>
@@ -2448,13 +2451,13 @@
     </row>
     <row r="113" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D113" s="1" t="s">
         <v>18</v>
@@ -2462,13 +2465,13 @@
     </row>
     <row r="114" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D114" s="1" t="s">
         <v>18</v>
@@ -2476,7 +2479,7 @@
     </row>
     <row r="115" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B115" s="1" t="s">
         <v>8</v>
@@ -2490,7 +2493,7 @@
     </row>
     <row r="116" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B116" s="1" t="s">
         <v>5</v>
@@ -2504,7 +2507,7 @@
     </row>
     <row r="117" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B117" s="1" t="s">
         <v>10</v>
@@ -2518,7 +2521,7 @@
     </row>
     <row r="118" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B118" s="1" t="s">
         <v>12</v>
@@ -2532,69 +2535,69 @@
     </row>
     <row r="119" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D119" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B120" s="1" t="s">
         <v>31</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D120" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B121" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C121" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D121" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C122" s="7" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D122" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D123" s="1" t="s">
         <v>18</v>
@@ -2602,13 +2605,13 @@
     </row>
     <row r="124" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D124" s="1" t="s">
         <v>18</v>
@@ -2616,13 +2619,13 @@
     </row>
     <row r="125" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B125" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D125" s="1" t="s">
         <v>18</v>
@@ -2630,13 +2633,13 @@
     </row>
     <row r="126" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D126" s="1" t="s">
         <v>18</v>
@@ -2644,27 +2647,27 @@
     </row>
     <row r="127" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B127" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C127" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="D127" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="C127" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="D127" s="1" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B128" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D128" s="1" t="s">
         <v>18</v>
@@ -2672,27 +2675,27 @@
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B129" s="1" t="s">
         <v>26</v>
       </c>
       <c r="C129" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D129" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D130" s="1" t="s">
         <v>18</v>
@@ -2700,41 +2703,41 @@
     </row>
     <row r="131" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A131" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D131" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C132" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D132" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D133" s="1" t="s">
         <v>18</v>
@@ -2742,13 +2745,13 @@
     </row>
     <row r="134" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C134" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D134" s="1" t="s">
         <v>18</v>
@@ -2756,13 +2759,13 @@
     </row>
     <row r="135" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B135" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C135" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D135" s="1" t="s">
         <v>18</v>
@@ -2770,35 +2773,35 @@
     </row>
     <row r="136" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B136" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C136" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D136" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="C136" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D136" s="1" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B137" s="1" t="s">
         <v>26</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D137" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B138" s="1" t="s">
         <v>31</v>
@@ -2812,7 +2815,7 @@
     </row>
     <row r="139" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B139" s="1" t="s">
         <v>33</v>
@@ -2826,7 +2829,7 @@
     </row>
     <row r="140" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B140" s="1" t="s">
         <v>16</v>
@@ -2835,7 +2838,7 @@
         <v>17</v>
       </c>
       <c r="D140" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>